<commit_message>
[Excel+YAML] Update Excel version of OWASP Top 10 Web 2021 + Update YAML
Add ":2021" to Ref. IDs so we can differentiate them with the 2025 version.
</commit_message>
<xml_diff>
--- a/tools/excel/owasp/owasp-top-10-web.xlsx
+++ b/tools/excel/owasp/owasp-top-10-web.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\owasp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD143A72-53C0-47FF-A568-0DE1FE9A4553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CAA34EB-2A94-4A49-98A8-6F860F3D7BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37824" yWindow="-5628" windowWidth="28704" windowHeight="16668" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25284" yWindow="-4128" windowWidth="28704" windowHeight="16188" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="63">
   <si>
     <t>type</t>
   </si>
@@ -55,9 +55,6 @@
   </si>
   <si>
     <t>version</t>
-  </si>
-  <si>
-    <t>1</t>
   </si>
   <si>
     <t>provider</t>
@@ -182,6 +179,39 @@
   </si>
   <si>
     <t>OWASP-top-10-Web_2021</t>
+  </si>
+  <si>
+    <t>node_id</t>
+  </si>
+  <si>
+    <t>A01:2021</t>
+  </si>
+  <si>
+    <t>A02:2021</t>
+  </si>
+  <si>
+    <t>A03:2021</t>
+  </si>
+  <si>
+    <t>A04:2021</t>
+  </si>
+  <si>
+    <t>A05:2021</t>
+  </si>
+  <si>
+    <t>A06:2021</t>
+  </si>
+  <si>
+    <t>A07:2021</t>
+  </si>
+  <si>
+    <t>A08:2021</t>
+  </si>
+  <si>
+    <t>A09:2021</t>
+  </si>
+  <si>
+    <t>A10:2021</t>
   </si>
 </sst>
 </file>
@@ -229,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -239,6 +269,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -489,7 +522,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -497,7 +530,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -512,32 +545,32 @@
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>11</v>
+      <c r="B7" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="106.2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -559,15 +592,15 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -577,133 +610,167 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="100" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="40.200000000000003" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="53.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="53.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="4" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="66.599999999999994" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="66.599999999999994" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="4" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="27" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="4" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="106.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="106.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="4" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="119.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="119.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="4" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="27" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="4" t="s">
+    </row>
+    <row r="9" spans="1:4" ht="106.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="106.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="4" t="s">
+    </row>
+    <row r="10" spans="1:4" ht="27" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="27" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="4" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="66.599999999999994" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="66.599999999999994" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>